<commit_message>
refactor: consolidate and reorganize dataset structure by migrating raw and cleaned CSVs into a unified directory.
</commit_message>
<xml_diff>
--- a/batches/25/daily/day_02.xlsx
+++ b/batches/25/daily/day_02.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10325"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10330"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/ALI_2/work/acciojob/modules/sql/batches/25/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/ALI_2/work/acciojob/modules/sql/batches/25/daily/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26215F2C-017A-C848-92E4-E97EED17DACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53BEC6BB-17D7-354C-9151-DAE02A272AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="3" xr2:uid="{31D46116-0E5E-6C44-A535-E126D5B67C6E}"/>
+    <workbookView xWindow="29400" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="5" xr2:uid="{31D46116-0E5E-6C44-A535-E126D5B67C6E}"/>
   </bookViews>
   <sheets>
     <sheet name="Recap" sheetId="1" r:id="rId1"/>
     <sheet name="Agenda" sheetId="2" r:id="rId2"/>
     <sheet name="First_Table" sheetId="3" r:id="rId3"/>
     <sheet name="Drop Delete Truncate" sheetId="4" r:id="rId4"/>
+    <sheet name="DML" sheetId="5" r:id="rId5"/>
+    <sheet name="Summary" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
   <si>
     <t>Land</t>
   </si>
@@ -141,6 +143,45 @@
   </si>
   <si>
     <t>Deleting all</t>
+  </si>
+  <si>
+    <t>Employee</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>DEPT</t>
+  </si>
+  <si>
+    <t>SALARY</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>d1</t>
+  </si>
+  <si>
+    <t>d2</t>
+  </si>
+  <si>
+    <t>d3</t>
+  </si>
+  <si>
+    <t>I want to delete the salary of employee 3</t>
+  </si>
+  <si>
+    <t>Update employee set salary ='' where id =3</t>
   </si>
 </sst>
 </file>
@@ -156,12 +197,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="12">
@@ -299,12 +346,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -314,6 +359,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -713,8 +762,8 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>105840</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="9" name="Ink 8">
@@ -733,7 +782,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="9" name="Ink 8">
@@ -778,8 +827,8 @@
       <xdr:row>19</xdr:row>
       <xdr:rowOff>45200</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="21" name="Ink 20">
@@ -798,7 +847,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="21" name="Ink 20">
@@ -843,8 +892,8 @@
       <xdr:row>16</xdr:row>
       <xdr:rowOff>67280</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="22" name="Ink 21">
@@ -863,7 +912,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="22" name="Ink 21">
@@ -908,8 +957,8 @@
       <xdr:row>11</xdr:row>
       <xdr:rowOff>191200</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="29" name="Ink 28">
@@ -928,7 +977,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="29" name="Ink 28">
@@ -973,8 +1022,8 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>113760</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="34" name="Ink 33">
@@ -993,7 +1042,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="34" name="Ink 33">
@@ -1038,8 +1087,8 @@
       <xdr:row>15</xdr:row>
       <xdr:rowOff>29640</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="35" name="Ink 34">
@@ -1058,7 +1107,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="35" name="Ink 34">
@@ -1103,8 +1152,8 @@
       <xdr:row>22</xdr:row>
       <xdr:rowOff>123200</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="45" name="Ink 44">
@@ -1123,7 +1172,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="45" name="Ink 44">
@@ -1168,8 +1217,8 @@
       <xdr:row>24</xdr:row>
       <xdr:rowOff>117840</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="48" name="Ink 47">
@@ -1188,7 +1237,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="48" name="Ink 47">
@@ -1233,8 +1282,8 @@
       <xdr:row>22</xdr:row>
       <xdr:rowOff>4400</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="59" name="Ink 58">
@@ -1253,7 +1302,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="59" name="Ink 58">
@@ -1298,8 +1347,8 @@
       <xdr:row>19</xdr:row>
       <xdr:rowOff>96680</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="60" name="Ink 59">
@@ -1318,7 +1367,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="60" name="Ink 59">
@@ -1474,6 +1523,456 @@
         <a:xfrm>
           <a:off x="1651000" y="16256000"/>
           <a:ext cx="7772400" cy="2289544"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>187290</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B5B54FC1-A420-33D2-CB9B-E7851FA06D14}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="304800" y="203200"/>
+          <a:ext cx="7772400" cy="3032090"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>45085</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDD20D9F-B663-BD96-7756-06ED4596D426}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="304800" y="3454400"/>
+          <a:ext cx="7772400" cy="3702685"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>736600</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C122EE0-A73D-7931-9600-F86B71B69677}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="304800" y="10160000"/>
+          <a:ext cx="4864100" cy="330200"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>140208</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{10EEEAAF-079A-BE11-FB53-9882460B9FCF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="304800" y="10769600"/>
+          <a:ext cx="7772400" cy="5423408"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>25400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>311150</xdr:colOff>
+      <xdr:row>113</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA66B46A-6D3E-42DC-0340-F4543958C664}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="323850" y="16687800"/>
+          <a:ext cx="5245100" cy="6311900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>114</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>144</xdr:row>
+      <xdr:rowOff>197441</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9BAD19BA-8CCE-5E21-793B-CC395C6F1D6F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="304800" y="23164800"/>
+          <a:ext cx="7772400" cy="6293441"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>146</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>155</xdr:row>
+      <xdr:rowOff>14584</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F852CB57-D42D-23F6-F21F-A3B265259575}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="304800" y="29667200"/>
+          <a:ext cx="7772400" cy="1843384"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>156</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>177</xdr:row>
+      <xdr:rowOff>157576</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6951B27E-088E-8D71-78A8-2DDA83B5C535}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="304800" y="31699200"/>
+          <a:ext cx="7772400" cy="4424776"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>29117</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{84C1F281-AD3C-AD33-7E68-1E73C3750C1B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="203200"/>
+          <a:ext cx="7772400" cy="5718717"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>131956</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28473A5D-537D-C0A1-C8FF-AD26DEA4AB39}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="6096000"/>
+          <a:ext cx="7772400" cy="4602356"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2187,15 +2686,14 @@
       <c r="J66" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K66" s="5" t="s">
+      <c r="K66" t="s">
         <v>15</v>
       </c>
-      <c r="L66" s="6"/>
+      <c r="L66" s="5"/>
     </row>
     <row r="67" spans="9:12" x14ac:dyDescent="0.2">
       <c r="J67" s="4"/>
-      <c r="K67" s="5"/>
-      <c r="L67" s="6"/>
+      <c r="L67" s="5"/>
     </row>
     <row r="68" spans="9:12" x14ac:dyDescent="0.2">
       <c r="I68" t="s">
@@ -2204,40 +2702,39 @@
       <c r="J68" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K68" s="5" t="s">
+      <c r="K68" t="s">
         <v>14</v>
       </c>
-      <c r="L68" s="6"/>
+      <c r="L68" s="5"/>
     </row>
     <row r="69" spans="9:12" x14ac:dyDescent="0.2">
       <c r="I69" t="s">
         <v>13</v>
       </c>
       <c r="J69" s="4"/>
-      <c r="K69" s="10" t="s">
+      <c r="K69" t="s">
         <v>16</v>
       </c>
-      <c r="L69" s="6"/>
+      <c r="L69" s="5"/>
     </row>
     <row r="70" spans="9:12" x14ac:dyDescent="0.2">
       <c r="I70" t="s">
         <v>19</v>
       </c>
       <c r="J70" s="4"/>
-      <c r="K70" s="10" t="s">
+      <c r="K70" t="s">
         <v>18</v>
       </c>
-      <c r="L70" s="6"/>
+      <c r="L70" s="5"/>
     </row>
     <row r="71" spans="9:12" x14ac:dyDescent="0.2">
       <c r="J71" s="4"/>
-      <c r="K71" s="5"/>
-      <c r="L71" s="6"/>
+      <c r="L71" s="5"/>
     </row>
     <row r="72" spans="9:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="J72" s="7"/>
-      <c r="K72" s="8"/>
-      <c r="L72" s="9"/>
+      <c r="J72" s="6"/>
+      <c r="K72" s="7"/>
+      <c r="L72" s="8"/>
     </row>
     <row r="73" spans="9:12" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="74" spans="9:12" x14ac:dyDescent="0.2">
@@ -2247,40 +2744,39 @@
     </row>
     <row r="75" spans="9:12" x14ac:dyDescent="0.2">
       <c r="J75" s="4"/>
-      <c r="K75" s="5" t="s">
+      <c r="K75" t="s">
         <v>7</v>
       </c>
-      <c r="L75" s="6"/>
+      <c r="L75" s="5"/>
     </row>
     <row r="76" spans="9:12" x14ac:dyDescent="0.2">
       <c r="I76" t="s">
         <v>12</v>
       </c>
       <c r="J76" s="4"/>
-      <c r="K76" s="5"/>
-      <c r="L76" s="6"/>
+      <c r="L76" s="5"/>
     </row>
     <row r="77" spans="9:12" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="J77" s="7"/>
-      <c r="K77" s="8"/>
-      <c r="L77" s="9"/>
+      <c r="J77" s="6"/>
+      <c r="K77" s="7"/>
+      <c r="L77" s="8"/>
     </row>
     <row r="80" spans="9:12" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="81" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="11" t="s">
+      <c r="B81" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C81" s="12"/>
-      <c r="D81" s="12"/>
-      <c r="E81" s="12"/>
-      <c r="F81" s="12"/>
-      <c r="G81" s="12"/>
-      <c r="H81" s="12"/>
-      <c r="I81" s="12"/>
-      <c r="J81" s="12"/>
-      <c r="K81" s="12"/>
-      <c r="L81" s="12"/>
-      <c r="M81" s="13"/>
+      <c r="C81" s="10"/>
+      <c r="D81" s="10"/>
+      <c r="E81" s="10"/>
+      <c r="F81" s="10"/>
+      <c r="G81" s="10"/>
+      <c r="H81" s="10"/>
+      <c r="I81" s="10"/>
+      <c r="J81" s="10"/>
+      <c r="K81" s="10"/>
+      <c r="L81" s="10"/>
+      <c r="M81" s="11"/>
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
@@ -2309,255 +2805,136 @@
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B83" s="4"/>
-      <c r="C83" s="5"/>
-      <c r="D83" s="6"/>
-      <c r="E83" s="5"/>
-      <c r="F83" s="5"/>
-      <c r="G83" s="5"/>
+      <c r="D83" s="5"/>
       <c r="H83" s="4"/>
-      <c r="I83" s="5"/>
-      <c r="J83" s="6"/>
-      <c r="K83" s="5"/>
-      <c r="L83" s="5"/>
-      <c r="M83" s="6"/>
+      <c r="J83" s="5"/>
+      <c r="M83" s="5"/>
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B84" s="4"/>
-      <c r="C84" s="5"/>
-      <c r="D84" s="6"/>
-      <c r="E84" s="5"/>
-      <c r="F84" s="5"/>
-      <c r="G84" s="5"/>
+      <c r="D84" s="5"/>
       <c r="H84" s="4"/>
-      <c r="I84" s="5"/>
-      <c r="J84" s="6"/>
-      <c r="K84" s="5"/>
-      <c r="L84" s="5"/>
-      <c r="M84" s="6"/>
+      <c r="J84" s="5"/>
+      <c r="M84" s="5"/>
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B85" s="4"/>
-      <c r="C85" s="5"/>
-      <c r="D85" s="6"/>
-      <c r="E85" s="5"/>
-      <c r="F85" s="5"/>
-      <c r="G85" s="5"/>
+      <c r="D85" s="5"/>
       <c r="H85" s="4"/>
-      <c r="I85" s="5"/>
-      <c r="J85" s="6"/>
-      <c r="K85" s="5"/>
-      <c r="L85" s="5"/>
-      <c r="M85" s="6"/>
+      <c r="J85" s="5"/>
+      <c r="M85" s="5"/>
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B86" s="4"/>
-      <c r="C86" s="5"/>
-      <c r="D86" s="6"/>
-      <c r="E86" s="5"/>
-      <c r="F86" s="5"/>
-      <c r="G86" s="5"/>
+      <c r="D86" s="5"/>
       <c r="H86" s="4"/>
-      <c r="I86" s="5"/>
-      <c r="J86" s="6"/>
-      <c r="K86" s="5"/>
-      <c r="L86" s="5"/>
-      <c r="M86" s="6"/>
+      <c r="J86" s="5"/>
+      <c r="M86" s="5"/>
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B87" s="4"/>
-      <c r="C87" s="5"/>
-      <c r="D87" s="6"/>
-      <c r="E87" s="5"/>
-      <c r="F87" s="5"/>
-      <c r="G87" s="5"/>
+      <c r="D87" s="5"/>
       <c r="H87" s="4"/>
-      <c r="I87" s="5"/>
-      <c r="J87" s="6"/>
-      <c r="K87" s="5"/>
-      <c r="L87" s="5"/>
-      <c r="M87" s="6"/>
+      <c r="J87" s="5"/>
+      <c r="M87" s="5"/>
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B88" s="4"/>
-      <c r="C88" s="5"/>
-      <c r="D88" s="6"/>
-      <c r="E88" s="5"/>
-      <c r="F88" s="5"/>
-      <c r="G88" s="5"/>
+      <c r="D88" s="5"/>
       <c r="H88" s="4"/>
-      <c r="I88" s="5"/>
-      <c r="J88" s="6"/>
-      <c r="K88" s="5"/>
-      <c r="L88" s="5"/>
-      <c r="M88" s="6"/>
+      <c r="J88" s="5"/>
+      <c r="M88" s="5"/>
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B89" s="4"/>
-      <c r="C89" s="5"/>
-      <c r="D89" s="6"/>
-      <c r="E89" s="5"/>
-      <c r="F89" s="5"/>
-      <c r="G89" s="5"/>
+      <c r="D89" s="5"/>
       <c r="H89" s="4"/>
-      <c r="I89" s="5"/>
-      <c r="J89" s="6"/>
-      <c r="K89" s="5"/>
-      <c r="L89" s="5"/>
-      <c r="M89" s="6"/>
+      <c r="J89" s="5"/>
+      <c r="M89" s="5"/>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B90" s="4"/>
-      <c r="C90" s="5"/>
-      <c r="D90" s="6"/>
-      <c r="E90" s="5"/>
-      <c r="F90" s="5"/>
-      <c r="G90" s="5"/>
+      <c r="D90" s="5"/>
       <c r="H90" s="4"/>
-      <c r="I90" s="5"/>
-      <c r="J90" s="6"/>
-      <c r="K90" s="5"/>
-      <c r="L90" s="5"/>
-      <c r="M90" s="6"/>
+      <c r="J90" s="5"/>
+      <c r="M90" s="5"/>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B91" s="4"/>
-      <c r="C91" s="5"/>
-      <c r="D91" s="6"/>
-      <c r="E91" s="5"/>
-      <c r="F91" s="5"/>
-      <c r="G91" s="5"/>
+      <c r="D91" s="5"/>
       <c r="H91" s="4"/>
-      <c r="I91" s="5"/>
-      <c r="J91" s="6"/>
-      <c r="K91" s="5"/>
-      <c r="L91" s="5"/>
-      <c r="M91" s="6"/>
+      <c r="J91" s="5"/>
+      <c r="M91" s="5"/>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B92" s="4"/>
-      <c r="C92" s="5"/>
-      <c r="D92" s="6"/>
-      <c r="E92" s="5"/>
-      <c r="F92" s="5"/>
-      <c r="G92" s="5"/>
+      <c r="D92" s="5"/>
       <c r="H92" s="4"/>
-      <c r="I92" s="5"/>
-      <c r="J92" s="6"/>
-      <c r="K92" s="5"/>
-      <c r="L92" s="5"/>
-      <c r="M92" s="6"/>
+      <c r="J92" s="5"/>
+      <c r="M92" s="5"/>
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B93" s="4"/>
-      <c r="C93" s="5"/>
-      <c r="D93" s="6"/>
-      <c r="E93" s="5"/>
-      <c r="F93" s="5"/>
-      <c r="G93" s="5"/>
+      <c r="D93" s="5"/>
       <c r="H93" s="4"/>
-      <c r="I93" s="5"/>
-      <c r="J93" s="6"/>
-      <c r="K93" s="5"/>
-      <c r="L93" s="5"/>
-      <c r="M93" s="6"/>
+      <c r="J93" s="5"/>
+      <c r="M93" s="5"/>
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B94" s="4"/>
-      <c r="C94" s="5"/>
-      <c r="D94" s="6"/>
-      <c r="E94" s="5"/>
-      <c r="F94" s="5"/>
-      <c r="G94" s="5"/>
+      <c r="D94" s="5"/>
       <c r="H94" s="4"/>
-      <c r="I94" s="5"/>
-      <c r="J94" s="6"/>
-      <c r="K94" s="5"/>
-      <c r="L94" s="5"/>
-      <c r="M94" s="6"/>
+      <c r="J94" s="5"/>
+      <c r="M94" s="5"/>
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B95" s="4"/>
-      <c r="C95" s="5"/>
-      <c r="D95" s="6"/>
-      <c r="E95" s="5"/>
-      <c r="F95" s="5"/>
-      <c r="G95" s="5"/>
+      <c r="D95" s="5"/>
       <c r="H95" s="4"/>
-      <c r="I95" s="5"/>
-      <c r="J95" s="6"/>
-      <c r="K95" s="5"/>
-      <c r="L95" s="5"/>
-      <c r="M95" s="6"/>
+      <c r="J95" s="5"/>
+      <c r="M95" s="5"/>
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.2">
       <c r="B96" s="4"/>
-      <c r="C96" s="5"/>
-      <c r="D96" s="6"/>
-      <c r="E96" s="5"/>
-      <c r="F96" s="5"/>
-      <c r="G96" s="5"/>
+      <c r="D96" s="5"/>
       <c r="H96" s="4"/>
-      <c r="I96" s="5"/>
-      <c r="J96" s="6"/>
-      <c r="K96" s="5"/>
-      <c r="L96" s="5"/>
-      <c r="M96" s="6"/>
+      <c r="J96" s="5"/>
+      <c r="M96" s="5"/>
     </row>
     <row r="97" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B97" s="4"/>
-      <c r="C97" s="5"/>
-      <c r="D97" s="6"/>
-      <c r="E97" s="5"/>
-      <c r="F97" s="5"/>
-      <c r="G97" s="5"/>
+      <c r="D97" s="5"/>
       <c r="H97" s="4"/>
-      <c r="I97" s="5"/>
-      <c r="J97" s="6"/>
-      <c r="K97" s="5"/>
-      <c r="L97" s="5"/>
-      <c r="M97" s="6"/>
+      <c r="J97" s="5"/>
+      <c r="M97" s="5"/>
     </row>
     <row r="98" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B98" s="4"/>
-      <c r="C98" s="5"/>
-      <c r="D98" s="6"/>
-      <c r="E98" s="5"/>
-      <c r="F98" s="5"/>
-      <c r="G98" s="5"/>
+      <c r="D98" s="5"/>
       <c r="H98" s="4"/>
-      <c r="I98" s="5"/>
-      <c r="J98" s="6"/>
-      <c r="K98" s="5"/>
-      <c r="L98" s="5"/>
-      <c r="M98" s="6"/>
+      <c r="J98" s="5"/>
+      <c r="M98" s="5"/>
     </row>
     <row r="99" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B99" s="4"/>
-      <c r="C99" s="5"/>
-      <c r="D99" s="6"/>
-      <c r="E99" s="5"/>
-      <c r="F99" s="5"/>
-      <c r="G99" s="5"/>
+      <c r="D99" s="5"/>
       <c r="H99" s="4"/>
-      <c r="I99" s="5"/>
-      <c r="J99" s="6"/>
-      <c r="K99" s="5"/>
-      <c r="L99" s="5"/>
-      <c r="M99" s="6"/>
+      <c r="J99" s="5"/>
+      <c r="M99" s="5"/>
     </row>
     <row r="100" spans="2:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B100" s="7"/>
-      <c r="C100" s="8"/>
-      <c r="D100" s="9"/>
-      <c r="E100" s="8"/>
-      <c r="F100" s="8"/>
-      <c r="G100" s="8"/>
-      <c r="H100" s="7"/>
-      <c r="I100" s="8"/>
-      <c r="J100" s="9"/>
-      <c r="K100" s="8"/>
-      <c r="L100" s="8"/>
-      <c r="M100" s="9"/>
+      <c r="B100" s="6"/>
+      <c r="C100" s="7"/>
+      <c r="D100" s="8"/>
+      <c r="E100" s="7"/>
+      <c r="F100" s="7"/>
+      <c r="G100" s="7"/>
+      <c r="H100" s="6"/>
+      <c r="I100" s="7"/>
+      <c r="J100" s="8"/>
+      <c r="K100" s="7"/>
+      <c r="L100" s="7"/>
+      <c r="M100" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2621,4 +2998,164 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74F1B189-E113-834F-957C-4DA2D6B8B5F1}">
+  <dimension ref="B37:J48"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C39" t="s">
+        <v>34</v>
+      </c>
+      <c r="D39" t="s">
+        <v>35</v>
+      </c>
+      <c r="E39" t="s">
+        <v>36</v>
+      </c>
+      <c r="F39" t="s">
+        <v>37</v>
+      </c>
+      <c r="H39" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="I39" s="12"/>
+      <c r="J39" s="12"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C40">
+        <v>1</v>
+      </c>
+      <c r="D40" t="s">
+        <v>38</v>
+      </c>
+      <c r="E40" t="s">
+        <v>41</v>
+      </c>
+      <c r="F40">
+        <v>1000</v>
+      </c>
+      <c r="H40" s="12"/>
+      <c r="I40" s="12"/>
+      <c r="J40" s="12"/>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41" t="s">
+        <v>39</v>
+      </c>
+      <c r="E41" t="s">
+        <v>42</v>
+      </c>
+      <c r="F41">
+        <v>2000</v>
+      </c>
+      <c r="H41" s="12"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="12"/>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C42" s="13">
+        <v>3</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E42" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F42" s="13">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="H43" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C45" t="s">
+        <v>34</v>
+      </c>
+      <c r="D45" t="s">
+        <v>35</v>
+      </c>
+      <c r="E45" t="s">
+        <v>36</v>
+      </c>
+      <c r="F45" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C46">
+        <v>1</v>
+      </c>
+      <c r="D46" t="s">
+        <v>38</v>
+      </c>
+      <c r="E46" t="s">
+        <v>41</v>
+      </c>
+      <c r="F46">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C47">
+        <v>2</v>
+      </c>
+      <c r="D47" t="s">
+        <v>39</v>
+      </c>
+      <c r="E47" t="s">
+        <v>42</v>
+      </c>
+      <c r="F47">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C48">
+        <v>3</v>
+      </c>
+      <c r="D48" t="s">
+        <v>40</v>
+      </c>
+      <c r="E48" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="H39:J41"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA39192A-F75D-754C-87B1-912BC4640DF7}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>